<commit_message>
feat(import): téléphone facultatif et montant 0 accepté
- Import et modèle : téléphone client facultatif ; montant 0 accepté (négatif ou vide refusé)
- Formulaire de paiement et modification d'encaissement : montant 0 accepté

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/management/modele_import_clients_paiements.xlsx
+++ b/public/management/modele_import_clients_paiements.xlsx
@@ -240,7 +240,7 @@
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Ex. 0673125999</t>
+        <t>Ex. 0673125999 — facultatif. Sans téléphone, le client ne peut pas être reconnu s'il existe déjà dans l'application.</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
@@ -295,7 +295,7 @@
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Nombre, sans « DH ».</t>
+        <t>Nombre, sans « DH ». 0 accepté (mois offert, assurance gratuite…).</t>
       </text>
     </comment>
   </commentList>
@@ -804,9 +804,9 @@
           <t>Nom *</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
-          <t>Téléphone *</t>
+          <t>Téléphone</t>
         </is>
       </c>
       <c r="E1" s="6" t="inlineStr">
@@ -59121,7 +59121,7 @@
     <dataValidation sqref="A5:A2004" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Réf inconnue" error="Cette référence n'existe pas dans la feuille Clients." type="list">
       <formula1>Clients!$A$3:$A$2002</formula1>
     </dataValidation>
-    <dataValidation sqref="F5:F2004" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Montant invalide" error="Saisissez un montant positif." type="decimal" operator="greaterThan">
+    <dataValidation sqref="F5:F2004" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Montant invalide" error="Saisissez un montant positif ou 0." type="decimal" operator="greaterThanOrEqual">
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation sqref="D5:D2004" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Date invalide" error="Saisissez une date JJ/MM/AAAA." type="date" operator="between">

</xml_diff>